<commit_message>
modified my soyab with new account
</commit_message>
<xml_diff>
--- a/bank.xlsx
+++ b/bank.xlsx
@@ -455,12 +455,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Password</t>
         </is>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2200</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="3">
@@ -561,12 +561,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Balance</t>
         </is>
@@ -579,7 +579,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>935</v>
+        <v>49309</v>
       </c>
     </row>
     <row r="3">

</xml_diff>